<commit_message>
Checkout test cases added
</commit_message>
<xml_diff>
--- a/com.Demowebshop/src/test/resources/TestData/DemowebshopTestData.xlsx
+++ b/com.Demowebshop/src/test/resources/TestData/DemowebshopTestData.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="84">
   <si>
     <t>First Name</t>
   </si>
@@ -230,6 +230,66 @@
   </si>
   <si>
     <t>KrishnaArora2587@testxp.com</t>
+  </si>
+  <si>
+    <t>DeepakArora2956@testxp.com</t>
+  </si>
+  <si>
+    <t>RajeevArora2178@testxp.com</t>
+  </si>
+  <si>
+    <t>KritiBhardwaj1384@testxp.com</t>
+  </si>
+  <si>
+    <t>PriyaKumar1404@testxp.com</t>
+  </si>
+  <si>
+    <t>RajeevVerma4058@testxp.com</t>
+  </si>
+  <si>
+    <t>RahulVerma1217@testxp.com</t>
+  </si>
+  <si>
+    <t>PriyaNautiyal6790@testxp.com</t>
+  </si>
+  <si>
+    <t>PoojaGoyal6359@testxp.com</t>
+  </si>
+  <si>
+    <t>RajeevBisht2551@testxp.com</t>
+  </si>
+  <si>
+    <t>RahulBhardwaj4406@testxp.com</t>
+  </si>
+  <si>
+    <t>PriyaVerma2077@testxp.com</t>
+  </si>
+  <si>
+    <t>PreetiArora1177@testxp.com</t>
+  </si>
+  <si>
+    <t>PranyaKumar8829@testxp.com</t>
+  </si>
+  <si>
+    <t>NainaArora5504@testxp.com</t>
+  </si>
+  <si>
+    <t>RahulSingh9893@testxp.com</t>
+  </si>
+  <si>
+    <t>PriyaKumar8722@testxp.com</t>
+  </si>
+  <si>
+    <t>PreetiBhardwaj7958@testxp.com</t>
+  </si>
+  <si>
+    <t>NainaBhardwaj7002@testxp.com</t>
+  </si>
+  <si>
+    <t>PriyaArora6901@testxp.com</t>
+  </si>
+  <si>
+    <t>NainaSharma994@testxp.com</t>
   </si>
 </sst>
 </file>
@@ -803,10 +863,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>